<commit_message>
feat: Add initial data, model configurations, tuning results, and a trained model for anomaly detection across multiple categories.
</commit_message>
<xml_diff>
--- a/data/reference/Сводная информация.xlsx
+++ b/data/reference/Сводная информация.xlsx
@@ -1,33 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Соли для ВШН\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\safae\alma_servie\data\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65BAEA0A-22B3-4114-BD78-EF30A362B709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF2F42A6-7B0A-4873-840C-2009ED71F5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BB3161D3-3B7B-4D46-A259-ADB2A2FDD4F0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{BB3161D3-3B7B-4D46-A259-ADB2A2FDD4F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -174,7 +168,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,6 +187,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -208,7 +208,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -264,17 +264,29 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -593,26 +605,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98D41B45-64EC-4A9F-8500-64078998A578}">
   <dimension ref="A3:N20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="21.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.90625" style="1"/>
+    <col min="2" max="2" width="21.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="78.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="21.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="6.81640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="21.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -656,7 +668,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -697,7 +709,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="144" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="145" x14ac:dyDescent="0.35">
       <c r="A5" s="11">
         <v>2</v>
       </c>
@@ -740,7 +752,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="11">
         <v>3</v>
       </c>
@@ -783,7 +795,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A7" s="11">
         <v>4</v>
       </c>
@@ -826,7 +838,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="11">
         <v>5</v>
       </c>
@@ -869,7 +881,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
         <v>6</v>
       </c>
@@ -916,7 +928,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="116" x14ac:dyDescent="0.35">
       <c r="A10" s="11">
         <v>7</v>
       </c>
@@ -959,212 +971,200 @@
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="7">
+    <row r="11" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="20">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="21">
         <v>45883.083333333336</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="21">
         <v>45885.083333333336</v>
       </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="8">
-        <v>45884.109027777777</v>
-      </c>
-      <c r="I11" s="8">
+      <c r="H11" s="21">
+        <v>45884.025694444441</v>
+      </c>
+      <c r="I11" s="21">
         <v>45884.115277777775</v>
       </c>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="9">
-        <f t="shared" si="0"/>
-        <v>3.1249999992724042E-3</v>
-      </c>
-      <c r="M11" s="10">
+      <c r="L11" s="22">
+        <f t="shared" si="0"/>
+        <v>4.4791666667151731E-2</v>
+      </c>
+      <c r="M11" s="23">
         <f t="shared" si="1"/>
-        <v>6.2499999985448085E-3</v>
-      </c>
-      <c r="N11" s="10">
+        <v>8.9583333334303461E-2</v>
+      </c>
+      <c r="N11" s="23">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="7">
+    <row r="12" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="20">
         <v>9</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="20">
         <v>524</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="21">
         <v>45817.083333333336</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="21">
         <v>45819.083333333336</v>
       </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="8">
-        <v>45817.901388888888</v>
-      </c>
-      <c r="I12" s="8">
+      <c r="H12" s="21">
+        <v>45817.818055555559</v>
+      </c>
+      <c r="I12" s="21">
         <v>45818.645833333336</v>
       </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="9">
-        <f t="shared" si="0"/>
-        <v>0.37222222222408163</v>
-      </c>
-      <c r="M12" s="10">
+      <c r="L12" s="22">
+        <f t="shared" si="0"/>
+        <v>0.41388888888832298</v>
+      </c>
+      <c r="M12" s="23">
         <f t="shared" si="1"/>
-        <v>0.74444444444816327</v>
-      </c>
-      <c r="N12" s="10">
+        <v>0.82777777777664596</v>
+      </c>
+      <c r="N12" s="23">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="7">
+    <row r="13" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="20">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="21">
         <v>45879.083333333336</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="21">
         <v>45880.083333333336</v>
       </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="8">
-        <v>45879.486111111109</v>
-      </c>
-      <c r="I13" s="8">
+      <c r="H13" s="21">
+        <v>45879.402777777781</v>
+      </c>
+      <c r="I13" s="21">
         <v>45879.892361111109</v>
       </c>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="9">
-        <f t="shared" si="0"/>
-        <v>0.40625</v>
-      </c>
-      <c r="M13" s="10">
+      <c r="L13" s="22">
+        <f t="shared" si="0"/>
+        <v>0.48958333332848269</v>
+      </c>
+      <c r="M13" s="23">
         <f t="shared" si="1"/>
-        <v>0.40625</v>
-      </c>
-      <c r="N13" s="10">
+        <v>0.48958333332848269</v>
+      </c>
+      <c r="N13" s="23">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="7">
+    <row r="14" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="20">
         <v>11</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="21">
         <v>45828.083333333336</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="21">
         <v>45830.083333333336</v>
       </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="8">
-        <v>45829.438888888886</v>
-      </c>
-      <c r="I14" s="8">
+      <c r="H14" s="21">
+        <v>45829.355555555558</v>
+      </c>
+      <c r="I14" s="21">
         <v>45829.987500000003</v>
       </c>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="9">
-        <f t="shared" si="0"/>
-        <v>0.27430555555838509</v>
-      </c>
-      <c r="M14" s="10">
+      <c r="L14" s="22">
+        <f t="shared" si="0"/>
+        <v>0.31597222222262644</v>
+      </c>
+      <c r="M14" s="23">
         <f t="shared" si="1"/>
-        <v>0.54861111111677019</v>
-      </c>
-      <c r="N14" s="10">
+        <v>0.63194444444525288</v>
+      </c>
+      <c r="N14" s="23">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="19">
+    <row r="15" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="24">
         <v>12</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="25">
         <v>45775.083333333336</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="25">
         <v>45784.083333333336</v>
       </c>
-      <c r="G15" s="19"/>
-      <c r="H15" s="20">
-        <v>45780.5625</v>
-      </c>
-      <c r="I15" s="20">
+      <c r="G15" s="24"/>
+      <c r="H15" s="25">
+        <v>45780.479166666664</v>
+      </c>
+      <c r="I15" s="25">
         <v>45784.083333333336</v>
       </c>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="9">
-        <f t="shared" si="0"/>
-        <v>0.39120370370397317</v>
-      </c>
-      <c r="M15" s="21">
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="22">
+        <f t="shared" si="0"/>
+        <v>0.40046296296350192</v>
+      </c>
+      <c r="M15" s="26">
         <f t="shared" si="1"/>
-        <v>3.5208333333357587</v>
-      </c>
-      <c r="N15" s="21">
+        <v>3.6041666666715173</v>
+      </c>
+      <c r="N15" s="26">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="7">
         <v>13</v>
       </c>
@@ -1205,7 +1205,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
         <v>14</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <v>15</v>
       </c>
@@ -1266,7 +1266,7 @@
         <v>45976.083333333336</v>
       </c>
       <c r="G18" s="15"/>
-      <c r="H18" s="22">
+      <c r="H18" s="19">
         <v>45952</v>
       </c>
       <c r="I18" s="16">
@@ -1287,7 +1287,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <v>16</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Add new pritok well data
</commit_message>
<xml_diff>
--- a/data/reference/Сводная информация.xlsx
+++ b/data/reference/Сводная информация.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\safae\alma_servie\data\reference\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ruslan_safaev\alma_servie\data\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19BFBAC-CD8B-4B9D-9CBD-ABDBED2484AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BDC9B1-F43F-473D-80D5-B5509AD8B364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{BB3161D3-3B7B-4D46-A259-ADB2A2FDD4F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="38">
   <si>
     <t>Месторождение</t>
   </si>
@@ -136,6 +136,12 @@
   </si>
   <si>
     <t>129л</t>
+  </si>
+  <si>
+    <t>5144г</t>
+  </si>
+  <si>
+    <t>Была остановка 03.03.2026 (игнорировать ее)</t>
   </si>
 </sst>
 </file>
@@ -145,7 +151,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,8 +173,35 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -177,29 +210,215 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFF2F5FA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF4CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D7E5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -208,84 +427,138 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -602,771 +875,1387 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="599" row="4">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{0A052928-C516-487A-B388-9D45956AC6F6}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;3c23a717-f32c-48d5-b395-3182ce7a3cd1&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98D41B45-64EC-4A9F-8500-64078998A578}">
-  <dimension ref="A3:N20"/>
+  <dimension ref="A2:N34"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="1"/>
-    <col min="2" max="2" width="21.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.6328125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="21.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.36328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.54296875" style="1" customWidth="1"/>
+    <col min="5" max="6" width="21.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="76.36328125" style="1" customWidth="1"/>
+    <col min="8" max="11" width="20.90625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="17.26953125" style="1" customWidth="1"/>
+    <col min="13" max="14" width="17.26953125" style="2" customWidth="1"/>
     <col min="15" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="2" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="1:14" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="31" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
+    <row r="4" spans="1:14" ht="91" x14ac:dyDescent="0.35">
+      <c r="A4" s="40">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="25">
         <v>45962.083333333336</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="25">
         <v>46023.083333333336</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="25">
         <v>45984</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="25">
         <v>46020.666666666664</v>
       </c>
-      <c r="L4" s="5">
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="26">
         <f>M4/N4</f>
         <v>0.60109289617482364</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="27">
         <f>I4-H4</f>
         <v>36.666666666664241</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="28">
         <f>F4-E4</f>
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="89.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11">
+    <row r="5" spans="1:14" ht="117" x14ac:dyDescent="0.35">
+      <c r="A5" s="41">
         <v>2</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="8">
         <v>3245</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="9">
         <v>45658.083333333336</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="9">
         <v>45789.083333333336</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="9">
         <v>45761.697222222225</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="9">
         <v>45789.083333333336</v>
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
-      <c r="L5" s="9">
-        <f t="shared" ref="L5:L20" si="0">M5/N5</f>
+      <c r="L5" s="10">
+        <f t="shared" ref="L5:L34" si="0">M5/N5</f>
         <v>0.20905428329092327</v>
       </c>
-      <c r="M5" s="10">
+      <c r="M5" s="11">
         <f t="shared" ref="M5:M18" si="1">I5-H5</f>
         <v>27.386111111110949</v>
       </c>
-      <c r="N5" s="10">
+      <c r="N5" s="21">
         <f t="shared" ref="N5:N18" si="2">F5-E5</f>
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="70.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11">
+    <row r="6" spans="1:14" ht="39" x14ac:dyDescent="0.35">
+      <c r="A6" s="42">
         <v>3</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="5">
         <v>45809.083333333336</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="5">
         <v>45836.083333333336</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="5">
         <v>45828.633333333331</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="5">
         <v>45836.083333333336</v>
       </c>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="9">
+      <c r="J6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="6">
         <f t="shared" si="0"/>
         <v>0.27592592592608761</v>
       </c>
-      <c r="M6" s="10">
+      <c r="M6" s="7">
         <f t="shared" si="1"/>
         <v>7.4500000000043656</v>
       </c>
-      <c r="N6" s="10">
+      <c r="N6" s="20">
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="60.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="11">
+    <row r="7" spans="1:14" ht="65" x14ac:dyDescent="0.35">
+      <c r="A7" s="41">
         <v>4</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="8">
         <v>3269</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="9">
         <v>45931.083333333336</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="9">
         <v>45959.083333333336</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="9">
         <v>45945.083333333336</v>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="9">
         <v>45957.489583333336</v>
       </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="9">
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="10">
         <f t="shared" si="0"/>
         <v>0.44308035714285715</v>
       </c>
-      <c r="M7" s="10">
+      <c r="M7" s="11">
         <f t="shared" si="1"/>
         <v>12.40625</v>
       </c>
-      <c r="N7" s="10">
+      <c r="N7" s="21">
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="93" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11">
+    <row r="8" spans="1:14" ht="39" x14ac:dyDescent="0.35">
+      <c r="A8" s="42">
         <v>5</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="4">
         <v>4039</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="5">
         <v>45748.083333333336</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="5">
         <v>45931.083333333336</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="5">
         <v>45806.458333333336</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="5">
         <v>45815.631944444445</v>
       </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="9">
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="6">
         <f t="shared" si="0"/>
         <v>5.0129022465079207E-2</v>
       </c>
-      <c r="M8" s="10">
+      <c r="M8" s="7">
         <f t="shared" si="1"/>
         <v>9.1736111111094942</v>
       </c>
-      <c r="N8" s="10">
+      <c r="N8" s="20">
         <f t="shared" si="2"/>
         <v>183</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11">
+    <row r="9" spans="1:14" ht="65" x14ac:dyDescent="0.35">
+      <c r="A9" s="41">
         <v>6</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="8">
         <v>408</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="9">
         <v>45748.083333333336</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="9">
         <v>45900.083333333336</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="9">
         <v>45810.194444444445</v>
       </c>
-      <c r="I9" s="12">
+      <c r="I9" s="9">
         <v>45834.472222222219</v>
       </c>
-      <c r="J9" s="12">
+      <c r="J9" s="9">
         <v>45860.791666666664</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="9">
         <v>45892.613888888889</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="10">
         <f t="shared" si="0"/>
         <v>0.15972222222219562</v>
       </c>
-      <c r="M9" s="10">
+      <c r="M9" s="11">
         <f t="shared" si="1"/>
         <v>24.277777777773736</v>
       </c>
-      <c r="N9" s="10">
+      <c r="N9" s="21">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11">
+    <row r="10" spans="1:14" ht="91" x14ac:dyDescent="0.35">
+      <c r="A10" s="42">
         <v>7</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="5">
         <v>45870.083333333336</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="5">
         <v>45968.083333333336</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="5">
         <v>45934.083333333336</v>
       </c>
-      <c r="I10" s="12">
+      <c r="I10" s="5">
         <v>45968.083333333336</v>
       </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="9">
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="6">
         <f t="shared" si="0"/>
         <v>0.34693877551020408</v>
       </c>
-      <c r="M10" s="10">
+      <c r="M10" s="7">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
-      <c r="N10" s="10">
+      <c r="N10" s="20">
         <f t="shared" si="2"/>
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="20">
+    <row r="11" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="41">
         <v>8</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="9">
         <v>45883.083333333336</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="9">
         <v>45885.083333333336</v>
       </c>
-      <c r="H11" s="21">
+      <c r="G11" s="36"/>
+      <c r="H11" s="9">
         <v>45884.025694444441</v>
       </c>
-      <c r="I11" s="21">
+      <c r="I11" s="9">
         <v>45884.115277777775</v>
       </c>
-      <c r="L11" s="22">
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="10">
         <f t="shared" si="0"/>
         <v>4.4791666667151731E-2</v>
       </c>
-      <c r="M11" s="23">
+      <c r="M11" s="11">
         <f t="shared" si="1"/>
         <v>8.9583333334303461E-2</v>
       </c>
-      <c r="N11" s="23">
+      <c r="N11" s="21">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="20">
+    <row r="12" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="42">
         <v>9</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="4">
         <v>524</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="5">
         <v>45817.083333333336</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="5">
         <v>45819.083333333336</v>
       </c>
-      <c r="H12" s="21">
+      <c r="G12" s="37"/>
+      <c r="H12" s="5">
         <v>45817.818055555559</v>
       </c>
-      <c r="I12" s="21">
+      <c r="I12" s="5">
         <v>45818.645833333336</v>
       </c>
-      <c r="L12" s="22">
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="6">
         <f t="shared" si="0"/>
         <v>0.41388888888832298</v>
       </c>
-      <c r="M12" s="23">
+      <c r="M12" s="7">
         <f t="shared" si="1"/>
         <v>0.82777777777664596</v>
       </c>
-      <c r="N12" s="23">
+      <c r="N12" s="20">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="20">
+    <row r="13" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="41">
         <v>10</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="9">
         <v>45879.083333333336</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="9">
         <v>45880.083333333336</v>
       </c>
-      <c r="H13" s="21">
+      <c r="G13" s="36"/>
+      <c r="H13" s="9">
         <v>45879.402777777781</v>
       </c>
-      <c r="I13" s="21">
+      <c r="I13" s="9">
         <v>45879.892361111109</v>
       </c>
-      <c r="L13" s="22">
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="10">
         <f t="shared" si="0"/>
         <v>0.48958333332848269</v>
       </c>
-      <c r="M13" s="23">
+      <c r="M13" s="11">
         <f t="shared" si="1"/>
         <v>0.48958333332848269</v>
       </c>
-      <c r="N13" s="23">
+      <c r="N13" s="21">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="20">
+    <row r="14" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="42">
         <v>11</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="5">
         <v>45828.083333333336</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="5">
         <v>45830.083333333336</v>
       </c>
-      <c r="H14" s="21">
+      <c r="G14" s="37"/>
+      <c r="H14" s="5">
         <v>45829.355555555558</v>
       </c>
-      <c r="I14" s="21">
+      <c r="I14" s="5">
         <v>45829.987500000003</v>
       </c>
-      <c r="L14" s="22">
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="6">
         <f t="shared" si="0"/>
         <v>0.31597222222262644</v>
       </c>
-      <c r="M14" s="23">
+      <c r="M14" s="7">
         <f t="shared" si="1"/>
         <v>0.63194444444525288</v>
       </c>
-      <c r="N14" s="23">
+      <c r="N14" s="20">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:14" s="20" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="24">
+    <row r="15" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="41">
         <v>12</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="9">
         <v>45775.083333333336</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="9">
         <v>45784.083333333336</v>
       </c>
-      <c r="G15" s="24"/>
-      <c r="H15" s="25">
+      <c r="G15" s="36"/>
+      <c r="H15" s="9">
         <v>45780.479166666664</v>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="9">
         <v>45784.083333333336</v>
       </c>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="22">
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="10">
         <f t="shared" si="0"/>
         <v>0.40046296296350192</v>
       </c>
-      <c r="M15" s="26">
+      <c r="M15" s="11">
         <f t="shared" si="1"/>
         <v>3.6041666666715173</v>
       </c>
-      <c r="N15" s="26">
+      <c r="N15" s="21">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A16" s="7">
+      <c r="A16" s="42">
         <v>13</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="4">
         <v>3261</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="5">
         <v>45931.083333333336</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="5">
         <v>45966.083333333336</v>
       </c>
-      <c r="G16" s="7"/>
-      <c r="H16" s="14">
+      <c r="G16" s="37"/>
+      <c r="H16" s="15">
         <v>45953</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="5">
         <v>45966.083333333336</v>
       </c>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="9">
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="6">
         <f t="shared" si="0"/>
         <v>0.37380952380959309</v>
       </c>
-      <c r="M16" s="10">
+      <c r="M16" s="7">
         <f t="shared" si="1"/>
         <v>13.083333333335759</v>
       </c>
-      <c r="N16" s="10">
+      <c r="N16" s="20">
         <f t="shared" si="2"/>
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A17" s="7">
+      <c r="A17" s="41">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="8">
         <v>495</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="9">
         <v>45922.083333333336</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="9">
         <v>45947.083333333336</v>
       </c>
-      <c r="G17" s="7"/>
+      <c r="G17" s="36"/>
       <c r="H17" s="14">
         <v>45938</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="9">
         <v>45947.083333333336</v>
       </c>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="9">
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="10">
         <f t="shared" si="0"/>
         <v>0.36333333333343032</v>
       </c>
-      <c r="M17" s="10">
+      <c r="M17" s="11">
         <f t="shared" si="1"/>
         <v>9.0833333333357587</v>
       </c>
-      <c r="N17" s="10">
+      <c r="N17" s="21">
         <f t="shared" si="2"/>
         <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A18" s="15">
+      <c r="A18" s="43">
         <v>15</v>
       </c>
-      <c r="B18" s="15" t="s">
+      <c r="B18" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="32">
         <v>902</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="33">
         <v>45945.083333333336</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="33">
         <v>45976.083333333336</v>
       </c>
-      <c r="G18" s="15"/>
-      <c r="H18" s="19">
+      <c r="G18" s="38"/>
+      <c r="H18" s="34">
         <v>45952</v>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="33">
         <v>45976.083333333336</v>
       </c>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="17">
+      <c r="J18" s="32"/>
+      <c r="K18" s="32"/>
+      <c r="L18" s="12">
         <f t="shared" si="0"/>
         <v>0.77688172043018577</v>
       </c>
-      <c r="M18" s="18">
+      <c r="M18" s="13">
         <f t="shared" si="1"/>
         <v>24.083333333335759</v>
       </c>
-      <c r="N18" s="18">
+      <c r="N18" s="22">
         <f t="shared" si="2"/>
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A19" s="15">
+      <c r="A19" s="43">
         <v>16</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="33">
         <v>45988.083333333336</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="33">
         <v>46015.083333333336</v>
       </c>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16">
+      <c r="G19" s="38"/>
+      <c r="H19" s="33">
         <v>46002.166666666664</v>
       </c>
-      <c r="I19" s="16">
+      <c r="I19" s="33">
         <v>46015.083333333336</v>
       </c>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="17">
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="12">
         <f t="shared" si="0"/>
         <v>0.47839506172857471</v>
       </c>
-      <c r="M19" s="18">
-        <f t="shared" ref="M19:M20" si="3">I19-H19</f>
+      <c r="M19" s="13">
+        <f t="shared" ref="M19:M34" si="3">I19-H19</f>
         <v>12.916666666671517</v>
       </c>
-      <c r="N19" s="18">
-        <f t="shared" ref="N19:N20" si="4">F19-E19</f>
+      <c r="N19" s="22">
+        <f t="shared" ref="N19:N34" si="4">F19-E19</f>
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A20" s="15">
+      <c r="A20" s="43">
         <v>17</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="33">
         <v>45992.083333333336</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="33">
         <v>46054.083333333336</v>
       </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="16">
+      <c r="G20" s="38"/>
+      <c r="H20" s="33">
         <v>46032.083333333336</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="33">
         <v>46054.083333333336</v>
       </c>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="17">
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+      <c r="L20" s="12">
         <f t="shared" si="0"/>
         <v>0.35483870967741937</v>
       </c>
-      <c r="M20" s="18">
+      <c r="M20" s="13">
         <f t="shared" si="3"/>
         <v>22</v>
       </c>
-      <c r="N20" s="18">
+      <c r="N20" s="22">
         <f t="shared" si="4"/>
         <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" s="41">
+        <v>18</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="8">
+        <v>1756</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="14">
+        <v>45965</v>
+      </c>
+      <c r="F21" s="14">
+        <v>45981</v>
+      </c>
+      <c r="G21" s="36"/>
+      <c r="H21" s="14">
+        <v>45972</v>
+      </c>
+      <c r="I21" s="14">
+        <v>45981</v>
+      </c>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="10">
+        <f t="shared" si="0"/>
+        <v>0.5625</v>
+      </c>
+      <c r="M21" s="11">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="N21" s="21">
+        <f t="shared" si="4"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A22" s="42">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="4">
+        <v>816</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="15">
+        <v>46023</v>
+      </c>
+      <c r="F22" s="15">
+        <v>46036</v>
+      </c>
+      <c r="G22" s="37"/>
+      <c r="H22" s="15">
+        <v>46032</v>
+      </c>
+      <c r="I22" s="15">
+        <v>46036</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="6">
+        <f t="shared" si="0"/>
+        <v>0.30769230769230771</v>
+      </c>
+      <c r="M22" s="7">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="N22" s="20">
+        <f t="shared" si="4"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A23" s="41">
+        <v>20</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="8">
+        <v>1809</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" s="14">
+        <v>46016</v>
+      </c>
+      <c r="F23" s="14">
+        <v>46047</v>
+      </c>
+      <c r="G23" s="36"/>
+      <c r="H23" s="14">
+        <v>46035</v>
+      </c>
+      <c r="I23" s="14">
+        <v>46047</v>
+      </c>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="10">
+        <f t="shared" si="0"/>
+        <v>0.38709677419354838</v>
+      </c>
+      <c r="M23" s="11">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="N23" s="21">
+        <f t="shared" si="4"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" s="42">
+        <v>21</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="4">
+        <v>792</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="15">
+        <v>45997</v>
+      </c>
+      <c r="F24" s="15">
+        <v>46039</v>
+      </c>
+      <c r="G24" s="37"/>
+      <c r="H24" s="15">
+        <v>46024</v>
+      </c>
+      <c r="I24" s="15">
+        <v>46039</v>
+      </c>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="6">
+        <f t="shared" si="0"/>
+        <v>0.35714285714285715</v>
+      </c>
+      <c r="M24" s="7">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="N24" s="20">
+        <f t="shared" si="4"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A25" s="41">
+        <v>22</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="8">
+        <v>1062</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" s="14">
+        <v>45998</v>
+      </c>
+      <c r="F25" s="14">
+        <v>46049</v>
+      </c>
+      <c r="G25" s="36"/>
+      <c r="H25" s="14">
+        <v>46024</v>
+      </c>
+      <c r="I25" s="14">
+        <v>46049</v>
+      </c>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="10">
+        <f t="shared" si="0"/>
+        <v>0.49019607843137253</v>
+      </c>
+      <c r="M25" s="11">
+        <f t="shared" si="3"/>
+        <v>25</v>
+      </c>
+      <c r="N25" s="21">
+        <f t="shared" si="4"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A26" s="42">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="4">
+        <v>691</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="15">
+        <v>45987</v>
+      </c>
+      <c r="F26" s="15">
+        <v>46029</v>
+      </c>
+      <c r="G26" s="37"/>
+      <c r="H26" s="15">
+        <v>46000</v>
+      </c>
+      <c r="I26" s="15">
+        <v>46020</v>
+      </c>
+      <c r="J26" s="15">
+        <v>46024</v>
+      </c>
+      <c r="K26" s="15">
+        <v>46029</v>
+      </c>
+      <c r="L26" s="6">
+        <f t="shared" si="0"/>
+        <v>0.47619047619047616</v>
+      </c>
+      <c r="M26" s="7">
+        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="N26" s="20">
+        <f t="shared" si="4"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A27" s="41">
+        <v>24</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="8">
+        <v>713</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="14">
+        <v>46012</v>
+      </c>
+      <c r="F27" s="14">
+        <v>46039</v>
+      </c>
+      <c r="G27" s="36"/>
+      <c r="H27" s="14">
+        <v>46024</v>
+      </c>
+      <c r="I27" s="14">
+        <v>46039</v>
+      </c>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="10">
+        <f t="shared" si="0"/>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="M27" s="11">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="N27" s="21">
+        <f t="shared" si="4"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A28" s="42">
+        <v>25</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="4">
+        <v>790</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="15">
+        <v>46009</v>
+      </c>
+      <c r="F28" s="15">
+        <v>46039</v>
+      </c>
+      <c r="G28" s="37"/>
+      <c r="H28" s="15">
+        <v>46024</v>
+      </c>
+      <c r="I28" s="15">
+        <v>46039</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="6">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="M28" s="7">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="N28" s="20">
+        <f t="shared" si="4"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A29" s="41">
+        <v>26</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" s="14">
+        <v>45998</v>
+      </c>
+      <c r="F29" s="14">
+        <v>46060</v>
+      </c>
+      <c r="G29" s="36"/>
+      <c r="H29" s="14">
+        <v>46047</v>
+      </c>
+      <c r="I29" s="14">
+        <v>46060</v>
+      </c>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="10">
+        <f t="shared" si="0"/>
+        <v>0.20967741935483872</v>
+      </c>
+      <c r="M29" s="11">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="N29" s="21">
+        <f t="shared" si="4"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A30" s="42">
+        <v>27</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="4">
+        <v>1395</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="15">
+        <v>46037</v>
+      </c>
+      <c r="F30" s="15">
+        <v>46082</v>
+      </c>
+      <c r="G30" s="37"/>
+      <c r="H30" s="15">
+        <v>46041</v>
+      </c>
+      <c r="I30" s="15">
+        <v>46082</v>
+      </c>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="6">
+        <f t="shared" si="0"/>
+        <v>0.91111111111111109</v>
+      </c>
+      <c r="M30" s="7">
+        <f t="shared" si="3"/>
+        <v>41</v>
+      </c>
+      <c r="N30" s="20">
+        <f t="shared" si="4"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A31" s="41">
+        <v>28</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C31" s="8">
+        <v>3245</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" s="14">
+        <v>46067</v>
+      </c>
+      <c r="F31" s="14">
+        <v>46095</v>
+      </c>
+      <c r="G31" s="36"/>
+      <c r="H31" s="14">
+        <v>46084</v>
+      </c>
+      <c r="I31" s="14">
+        <v>46095</v>
+      </c>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="10">
+        <f t="shared" si="0"/>
+        <v>0.39285714285714285</v>
+      </c>
+      <c r="M31" s="11">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="N31" s="21">
+        <f t="shared" si="4"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A32" s="42">
+        <v>29</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C32" s="4">
+        <v>3027</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="15">
+        <v>46067</v>
+      </c>
+      <c r="F32" s="15">
+        <v>46095</v>
+      </c>
+      <c r="G32" s="37"/>
+      <c r="H32" s="15">
+        <v>46084</v>
+      </c>
+      <c r="I32" s="15">
+        <v>46095</v>
+      </c>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="6">
+        <f t="shared" si="0"/>
+        <v>0.39285714285714285</v>
+      </c>
+      <c r="M32" s="7">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="N32" s="20">
+        <f t="shared" si="4"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A33" s="41">
+        <v>30</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="8">
+        <v>610</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="14">
+        <v>46071</v>
+      </c>
+      <c r="F33" s="14">
+        <v>46104</v>
+      </c>
+      <c r="G33" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="H33" s="14">
+        <v>46085</v>
+      </c>
+      <c r="I33" s="14">
+        <v>46104</v>
+      </c>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="10">
+        <f t="shared" si="0"/>
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="M33" s="11">
+        <f t="shared" si="3"/>
+        <v>19</v>
+      </c>
+      <c r="N33" s="21">
+        <f t="shared" si="4"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="44">
+        <v>31</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="16">
+        <v>602</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="17">
+        <v>46004</v>
+      </c>
+      <c r="F34" s="17">
+        <v>46094</v>
+      </c>
+      <c r="G34" s="39"/>
+      <c r="H34" s="17">
+        <v>46045</v>
+      </c>
+      <c r="I34" s="17">
+        <v>46059</v>
+      </c>
+      <c r="J34" s="17">
+        <v>46071</v>
+      </c>
+      <c r="K34" s="17">
+        <v>46094</v>
+      </c>
+      <c r="L34" s="18">
+        <f t="shared" si="0"/>
+        <v>0.15555555555555556</v>
+      </c>
+      <c r="M34" s="19">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="N34" s="23">
+        <f t="shared" si="4"/>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>